<commit_message>
Deploying to gh-pages from @ Sameerakhan05/pdd-testing@4d2c5458b27c25b62b40673c28da6642771c4251 🚀
</commit_message>
<xml_diff>
--- a/reports/history/build-2/Execution_Summary.xlsx
+++ b/reports/history/build-2/Execution_Summary.xlsx
@@ -22,13 +22,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>1</t>
+    <t>2</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T06:54:04.206Z</t>
+    <t>2026-06-24T07:29:43.990Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>504</v>
+        <v>497</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>